<commit_message>
add flatchart to priceList
</commit_message>
<xml_diff>
--- a/גדות סקיי - מחירון 46.xlsx
+++ b/גדות סקיי - מחירון 46.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Windows.old\Users\Public\VUE\Diary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD9E6A3F-252D-42CA-90F1-AC4283A15ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1154DF1B-A0B3-4FD3-9EAF-5AA61AB735CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{025406CF-A7AE-4DE8-B584-23F180A0A057}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{025406CF-A7AE-4DE8-B584-23F180A0A057}"/>
   </bookViews>
   <sheets>
     <sheet name="price" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="35">
   <si>
     <t>צפון דרום מערב</t>
   </si>
@@ -93,20 +93,68 @@
     <t>balconyArea</t>
   </si>
   <si>
-    <t>eqvivalentArea</t>
-  </si>
-  <si>
     <t>flatPrice</t>
   </si>
   <si>
     <t>status</t>
+  </si>
+  <si>
+    <t>equivalentArea</t>
+  </si>
+  <si>
+    <t>flatChart</t>
+  </si>
+  <si>
+    <t>1wOl1UIGqdJg383_-c_cMTUG5yx0XgX5Z</t>
+  </si>
+  <si>
+    <t>1c6Y_hGyiTvVyhuMy44CV-ShhpyqrnZcm</t>
+  </si>
+  <si>
+    <t>1i9Dwo6yOEQYPZaDPqco4mFlGemCRZwHy</t>
+  </si>
+  <si>
+    <t>1i1LQdDPVwsK2mAMOCC1yt6hoNyQQ7wek</t>
+  </si>
+  <si>
+    <t>1iHD6GZGS2I9HpWNJOs4vcKaC2hjHuMUy</t>
+  </si>
+  <si>
+    <t>1iKWq6_Zp_It_3-0RcohzHAWGRddKo8Ts</t>
+  </si>
+  <si>
+    <t>16htn7tXBb5dWKDqBsJTeNwOLYMp34LI7</t>
+  </si>
+  <si>
+    <t>1iTjQM3aiUlwgG6_fbwrNUYpuN_ZDkmFy</t>
+  </si>
+  <si>
+    <t>1XTmCfRZFrb4plxUccn-KU3ighCjYsygO</t>
+  </si>
+  <si>
+    <t>1PoIh_SoauvSZlbEyCtSepca2Dsq8-HWY</t>
+  </si>
+  <si>
+    <t>1iLsgx_jcr8BK0rI7QSLBE1ZxSH4sv79x</t>
+  </si>
+  <si>
+    <t>1BAmtQzomAb5reMZCM9TwVlqqAPTqQezT</t>
+  </si>
+  <si>
+    <t>1rv-Fpl3VwW-bPCoDHaUNUOHr2ww5Z1wg</t>
+  </si>
+  <si>
+    <t>1KG08jfYI7haJ2fRYLg7BHwQDMA_VLf4O</t>
+  </si>
+  <si>
+    <t>15nwOf_XYXw322MH1ZJtcpMKB--5xkot_</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,6 +181,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -432,7 +486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -569,6 +623,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -804,15 +859,17 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L979"/>
+  <dimension ref="A1:M979"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" customWidth="1"/>
     <col min="2" max="2" width="7.7109375" customWidth="1"/>
-    <col min="3" max="12" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="12" width="14.42578125" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="59.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="49" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" s="49" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
         <v>7</v>
       </c>
@@ -841,16 +898,19 @@
         <v>15</v>
       </c>
       <c r="J1" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="25" t="s">
+      <c r="L1" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="L1" s="25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M1" s="25" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="34">
         <v>0</v>
       </c>
@@ -879,14 +939,17 @@
         <v>157</v>
       </c>
       <c r="J2" s="38">
-        <v>182.33333333333334</v>
+        <v>183</v>
       </c>
       <c r="K2" s="39">
         <v>4500000</v>
       </c>
       <c r="L2" s="40"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M2" s="50" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="26">
         <v>1</v>
       </c>
@@ -923,8 +986,11 @@
       <c r="L3" s="33" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M3" s="50" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <v>1</v>
       </c>
@@ -961,8 +1027,11 @@
       <c r="L4" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M4" s="50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <v>1</v>
       </c>
@@ -999,8 +1068,11 @@
       <c r="L5" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M5" s="50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="17">
         <v>1</v>
       </c>
@@ -1037,8 +1109,11 @@
       <c r="L6" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" s="50" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>2</v>
       </c>
@@ -1075,8 +1150,11 @@
       <c r="L7" s="14" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7" s="50" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <v>2</v>
       </c>
@@ -1113,8 +1191,11 @@
       <c r="L8" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8" s="50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <v>2</v>
       </c>
@@ -1151,8 +1232,11 @@
       <c r="L9" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M9" s="50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="17">
         <v>2</v>
       </c>
@@ -1189,8 +1273,11 @@
       <c r="L10" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M10" s="50" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>3</v>
       </c>
@@ -1227,8 +1314,11 @@
       <c r="L11" s="14" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M11" s="50" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <v>3</v>
       </c>
@@ -1265,8 +1355,11 @@
       <c r="L12" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M12" s="50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <v>3</v>
       </c>
@@ -1303,8 +1396,11 @@
       <c r="L13" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M13" s="50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="17">
         <v>3</v>
       </c>
@@ -1341,8 +1437,11 @@
       <c r="L14" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M14" s="50" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>4</v>
       </c>
@@ -1377,8 +1476,11 @@
         <v>2485000</v>
       </c>
       <c r="L15" s="14"/>
-    </row>
-    <row r="16" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M15" s="50" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <v>4</v>
       </c>
@@ -1413,8 +1515,11 @@
         <v>2450000</v>
       </c>
       <c r="L16" s="16"/>
-    </row>
-    <row r="17" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M16" s="50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <v>4</v>
       </c>
@@ -1451,8 +1556,11 @@
       <c r="L17" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M17" s="50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="17">
         <v>4</v>
       </c>
@@ -1489,8 +1597,11 @@
       <c r="L18" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M18" s="50" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7">
         <v>5</v>
       </c>
@@ -1525,8 +1636,11 @@
         <v>2525000</v>
       </c>
       <c r="L19" s="14"/>
-    </row>
-    <row r="20" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M19" s="50" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <v>5</v>
       </c>
@@ -1561,8 +1675,11 @@
         <v>2490000</v>
       </c>
       <c r="L20" s="16"/>
-    </row>
-    <row r="21" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M20" s="50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <v>5</v>
       </c>
@@ -1599,8 +1716,11 @@
       <c r="L21" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M21" s="50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="17">
         <v>5</v>
       </c>
@@ -1637,8 +1757,11 @@
       <c r="L22" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M22" s="50" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7">
         <v>6</v>
       </c>
@@ -1673,8 +1796,11 @@
         <v>2565000</v>
       </c>
       <c r="L23" s="14"/>
-    </row>
-    <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M23" s="50" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <v>6</v>
       </c>
@@ -1709,8 +1835,11 @@
         <v>2530000</v>
       </c>
       <c r="L24" s="16"/>
-    </row>
-    <row r="25" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M24" s="50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <v>6</v>
       </c>
@@ -1745,8 +1874,11 @@
         <v>2792000</v>
       </c>
       <c r="L25" s="16"/>
-    </row>
-    <row r="26" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M25" s="50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="17">
         <v>6</v>
       </c>
@@ -1781,8 +1913,11 @@
         <v>2504000</v>
       </c>
       <c r="L26" s="24"/>
-    </row>
-    <row r="27" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M26" s="50" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7">
         <v>7</v>
       </c>
@@ -1817,8 +1952,11 @@
         <v>2605000</v>
       </c>
       <c r="L27" s="14"/>
-    </row>
-    <row r="28" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M27" s="50" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <v>7</v>
       </c>
@@ -1853,8 +1991,11 @@
         <v>2570000</v>
       </c>
       <c r="L28" s="16"/>
-    </row>
-    <row r="29" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M28" s="50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
         <v>7</v>
       </c>
@@ -1891,8 +2032,11 @@
       <c r="L29" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M29" s="50" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="41">
         <v>7</v>
       </c>
@@ -1927,8 +2071,11 @@
         <v>2592000</v>
       </c>
       <c r="L30" s="48"/>
-    </row>
-    <row r="31" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M30" s="50" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7">
         <v>8</v>
       </c>
@@ -1957,14 +2104,17 @@
         <v>55</v>
       </c>
       <c r="J31" s="12">
-        <v>138.33333333333334</v>
+        <v>139</v>
       </c>
       <c r="K31" s="13">
         <v>4200000</v>
       </c>
       <c r="L31" s="14"/>
-    </row>
-    <row r="32" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M31" s="50" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="17">
         <v>8</v>
       </c>
@@ -1999,8 +2149,11 @@
         <v>4500000</v>
       </c>
       <c r="L32" s="24"/>
-    </row>
-    <row r="33" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M32" s="50" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7">
         <v>0</v>
       </c>
@@ -2035,8 +2188,11 @@
         <v>4000000</v>
       </c>
       <c r="L33" s="14"/>
-    </row>
-    <row r="34" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M33" s="50" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="17">
         <v>0</v>
       </c>
@@ -2065,14 +2221,17 @@
         <v>187</v>
       </c>
       <c r="J34" s="22">
-        <v>147.33333333333334</v>
+        <v>148</v>
       </c>
       <c r="K34" s="23">
         <v>3900000</v>
       </c>
       <c r="L34" s="24"/>
-    </row>
-    <row r="35" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M34" s="50" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
         <v>1</v>
       </c>
@@ -2109,8 +2268,11 @@
       <c r="L35" s="14" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M35" s="50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15">
         <v>1</v>
       </c>
@@ -2147,8 +2309,11 @@
       <c r="L36" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M36" s="50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15">
         <v>1</v>
       </c>
@@ -2185,8 +2350,11 @@
       <c r="L37" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="38" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M37" s="50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="17">
         <v>1</v>
       </c>
@@ -2223,8 +2391,11 @@
       <c r="L38" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="39" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M38" s="50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7">
         <v>2</v>
       </c>
@@ -2261,8 +2432,11 @@
       <c r="L39" s="14" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="40" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M39" s="50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="15">
         <v>2</v>
       </c>
@@ -2299,8 +2473,11 @@
       <c r="L40" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="41" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M40" s="50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
         <v>2</v>
       </c>
@@ -2337,8 +2514,11 @@
       <c r="L41" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M41" s="50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="17">
         <v>2</v>
       </c>
@@ -2375,8 +2555,11 @@
       <c r="L42" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="43" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M42" s="50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7">
         <v>3</v>
       </c>
@@ -2411,8 +2594,11 @@
         <v>2648000</v>
       </c>
       <c r="L43" s="14"/>
-    </row>
-    <row r="44" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M43" s="50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="15">
         <v>3</v>
       </c>
@@ -2447,8 +2633,11 @@
         <v>2400000</v>
       </c>
       <c r="L44" s="16"/>
-    </row>
-    <row r="45" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M44" s="50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
         <v>3</v>
       </c>
@@ -2485,8 +2674,11 @@
       <c r="L45" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="46" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M45" s="50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="17">
         <v>3</v>
       </c>
@@ -2523,8 +2715,11 @@
       <c r="L46" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="47" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M46" s="50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
         <v>4</v>
       </c>
@@ -2559,8 +2754,11 @@
         <v>2688000</v>
       </c>
       <c r="L47" s="14"/>
-    </row>
-    <row r="48" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M47" s="50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="15">
         <v>4</v>
       </c>
@@ -2595,8 +2793,11 @@
         <v>2440000</v>
       </c>
       <c r="L48" s="16"/>
-    </row>
-    <row r="49" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M48" s="50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="15">
         <v>4</v>
       </c>
@@ -2633,8 +2834,11 @@
       <c r="L49" s="16" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="50" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M49" s="50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="17">
         <v>4</v>
       </c>
@@ -2671,8 +2875,11 @@
       <c r="L50" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="51" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M50" s="50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
         <v>5</v>
       </c>
@@ -2707,8 +2914,11 @@
         <v>2728000</v>
       </c>
       <c r="L51" s="14"/>
-    </row>
-    <row r="52" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M51" s="50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
         <v>5</v>
       </c>
@@ -2743,8 +2953,11 @@
         <v>2480000</v>
       </c>
       <c r="L52" s="16"/>
-    </row>
-    <row r="53" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M52" s="50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
         <v>5</v>
       </c>
@@ -2779,8 +2992,11 @@
         <v>2567000</v>
       </c>
       <c r="L53" s="16"/>
-    </row>
-    <row r="54" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M53" s="50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="17">
         <v>5</v>
       </c>
@@ -2817,8 +3033,11 @@
       <c r="L54" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="55" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M54" s="50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="7">
         <v>6</v>
       </c>
@@ -2853,8 +3072,11 @@
         <v>2768000</v>
       </c>
       <c r="L55" s="14"/>
-    </row>
-    <row r="56" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M55" s="50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
         <v>6</v>
       </c>
@@ -2889,8 +3111,11 @@
         <v>2520000</v>
       </c>
       <c r="L56" s="16"/>
-    </row>
-    <row r="57" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M56" s="50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
         <v>6</v>
       </c>
@@ -2925,8 +3150,11 @@
         <v>2607000</v>
       </c>
       <c r="L57" s="16"/>
-    </row>
-    <row r="58" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M57" s="50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="17">
         <v>6</v>
       </c>
@@ -2961,8 +3189,11 @@
         <v>2848000</v>
       </c>
       <c r="L58" s="24"/>
-    </row>
-    <row r="59" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M58" s="50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="7">
         <v>7</v>
       </c>
@@ -2997,8 +3228,11 @@
         <v>2906000</v>
       </c>
       <c r="L59" s="14"/>
-    </row>
-    <row r="60" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M59" s="50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="15">
         <v>7</v>
       </c>
@@ -3033,8 +3267,11 @@
         <v>2658000</v>
       </c>
       <c r="L60" s="16"/>
-    </row>
-    <row r="61" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M60" s="50" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="15">
         <v>7</v>
       </c>
@@ -3069,8 +3306,11 @@
         <v>2697000</v>
       </c>
       <c r="L61" s="16"/>
-    </row>
-    <row r="62" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M61" s="50" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="17">
         <v>7</v>
       </c>
@@ -3107,8 +3347,11 @@
       <c r="L62" s="24" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="63" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M62" s="50" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7">
         <v>8</v>
       </c>
@@ -3137,14 +3380,17 @@
         <v>64</v>
       </c>
       <c r="J63" s="12">
-        <v>141.33333333333334</v>
+        <v>142</v>
       </c>
       <c r="K63" s="13">
         <v>4200000</v>
       </c>
       <c r="L63" s="14"/>
-    </row>
-    <row r="64" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M63" s="50" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="17">
         <v>8</v>
       </c>
@@ -3173,12 +3419,15 @@
         <v>49</v>
       </c>
       <c r="J64" s="22">
-        <v>164.33333333333334</v>
+        <v>165</v>
       </c>
       <c r="K64" s="23">
         <v>4500000</v>
       </c>
       <c r="L64" s="24"/>
+      <c r="M64" s="50" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>